<commit_message>
prototype: Add sheet music for "Twinkle, Twinkle, Little Star" v1: 1. Add sheet music for "Twinkle, Twinkle, Little Star" 2. Update the screenplay
</commit_message>
<xml_diff>
--- a/v1/screenplay_zh.xlsx
+++ b/v1/screenplay_zh.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEV\project\self_playing_ruler\v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D36613-7CBA-4B03-8002-86AF23254340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B928CA9-3714-458F-9477-6C58C5B77891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-130" yWindow="-130" windowWidth="25860" windowHeight="13940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="封标" sheetId="4" r:id="rId1"/>
-    <sheet name="完整版" sheetId="1" r:id="rId2"/>
-    <sheet name="简洁版" sheetId="3" r:id="rId3"/>
-    <sheet name="素材引用" sheetId="5" r:id="rId4"/>
+    <sheet name="剧本" sheetId="1" r:id="rId2"/>
+    <sheet name="素材引用" sheetId="5" r:id="rId3"/>
+    <sheet name="雷达图制作" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="143">
   <si>
     <t>​​画面描述 (分镜)​​</t>
   </si>
@@ -81,10 +81,6 @@
   </si>
   <si>
     <t xml:space="preserve">​​时间戳 </t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>此前录制的慢放视频（使用类似进度条的东西，显示每部分时间占用）</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -184,14 +180,6 @@
   <si>
     <t>哆啦A梦掏出：钢尺</t>
     <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>手绘设计图展示
-每个器件特写气泡（根据口播节奏依次出现）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>演奏《哆啦A梦》</t>
   </si>
   <si>
     <t>（华强买瓜语音）</t>
@@ -270,16 +258,6 @@
   </si>
   <si>
     <t>口播出镜
-弹奏一个音+手机fft，浮现文字：误差xxx</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>口播出镜
-麦克风--&gt;开发板-(usb线)-&gt;mic--电脑</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>口播出镜
 展示一个串口谱子</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -290,11 +268,6 @@
   </si>
   <si>
     <t>演奏前：来看看效果吧！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>口播出镜
-演奏《哆啦A梦》</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -309,20 +282,6 @@
     <t>首先就是演奏速度比较慢
 慢速演奏完：这样已经是极限了
 如果调快速度就变成这样了！！这限制了它演奏很多快节奏的曲目</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>钢尺琴插入电源、插入数据线，按调音键调音（如果时间长就快进）
-mid键盘插入数据线
-打开宿主软件（先配置好，最小化），选择xxx设备
-使用MIDI键盘弹奏一小段音乐《欢乐颂》</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>夺舍钢尺
-口播出镜
-废弃的3d打印件
-100多个commit屏幕滚动</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -365,13 +324,6 @@
   </si>
   <si>
     <t>夺舍BGM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>夺舍（使用伤心欲茄声音AI合成）：斯你麻赛，nice什么呀！修改了多少个版本才有现在的效果的呀？你是nice了，我的刻度线都磨没了，八嘎压路！
-我：这不是考虑到观众老爷的观看体验，将中间的调试过程压缩了么
-我：结构上迭代设计了很多版
-我：代码也是改了很多次，这里有100多个commit</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -487,13 +439,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>还有一个问题，就是，乐谱的存储与传输
-原型机的谱子格式是自定义的：
-比如，("5#.", 1)：即表示高音升Sol，时长为一拍，用串口发送一个音符演奏一个音符
-这样，虽然调试方便，但每首歌都要一个音一个音来写，太麻烦了！！！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>10:19-10:32 https://www.bilibili.com/video/BV187411r7hp/</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -567,20 +512,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>todo：测试哆啦A梦的演奏效果</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>我：我一个程序员，让我弹钢尺，我能弹么？
-范志毅：“弹不了！没那个能力知道吧！”</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>过渡到:
-Cyberuler 2025</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>怎么办呢？那就…上！科！技！
 “自动演奏的钢尺”
 让我们开始吧</t>
@@ -588,16 +519,6 @@
   </si>
   <si>
     <t>加加鸽</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>TODO:需要制作片头</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>我先设计了一个原型机验证可行性
-模仿大佬演奏的动作，使用丝杆步进电机来精确控制钢尺移动、
-使用一个舵机压住钢尺、另一个舵机弹拨钢尺</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -705,12 +626,171 @@
     <t>取出模型--&gt;拿到工作台--&gt;掰下来 / 一个响指出现在桌面</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>sg90舵机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>42步进电机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>小无刷电机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>响应快</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>体积小</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>扭力大</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>演奏《小星星》</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">夺舍（使用伤心欲茄声音AI合成）：斯你麻赛，nice什么呀！修改了多少个版本才有现在的效果的呀？你是nice了，我的刻度线都磨没了，八嘎压路！
+我：这不是考虑到观众老爷的观看体验，将中间的调试过程压缩了么
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>我：结构上迭代设计了很多版，看，盒子里有好多
+我：代码也是改了很多次，这里有100多个commit</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>夺舍钢尺</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+口播出镜
+废弃的3d打印件
+100多个commit屏幕滚动</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>我：我一个程序员，让我弹钢尺，我能弹么？弹不了！
+范志毅：“没这个能力知道吧！”</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>过渡到:
+Cyberuler 2025，添加文本特效</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+原型机演奏《小星星》</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+自动弹奏一个音+手机fft，浮现文字：误差xxx</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>演奏一个音符的慢放视频（使用类似进度条的东西，显示每部分时间占用）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>我先设计了一个原型机验证可行性
+模仿演奏的动作，使用丝杆步进电机来精确控制钢尺移动、
+使用一个舵机压住钢尺、另一个舵机弹拨钢尺</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>手绘设计图展示</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（舵机、丝杆步进电机）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+每个器件特写气泡（根据口播节奏依次出现）</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+麦克风--&gt;开发板-(usb线)-&gt;mic--电脑
+添加一个DRI Mic的在音频设备中的截图</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>还有一个问题，就是，乐谱的存储与传输
+原型机的谱子格式是自定义的：
+比如，("5", 1)：即表示Sol，时长为一拍，用串口发送一个音符演奏一个音符
+这样，虽然调试方便，但每首歌都要一个音一个音来写，太麻烦了！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>；</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="等线"/>
@@ -776,6 +856,13 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -810,13 +897,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="1" tint="0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -911,7 +998,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -993,7 +1080,22 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="45" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="21" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1014,28 +1116,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="45" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="21" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="45" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="21" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="21" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="45" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1053,6 +1158,1040 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.44070841380676479"/>
+          <c:y val="0.16961546837213035"/>
+          <c:w val="0.5827211133492034"/>
+          <c:h val="0.7869142968699161"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>雷达图制作!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>sg90舵机</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>雷达图制作!$B$1:$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>响应快</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>体积小</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>扭力大</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>雷达图制作!$B$2:$D$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B37B-435F-A1A5-5285699195E0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>雷达图制作!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>小无刷电机</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>雷达图制作!$B$1:$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>响应快</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>体积小</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>扭力大</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>雷达图制作!$B$3:$D$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-B37B-435F-A1A5-5285699195E0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>雷达图制作!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>42步进电机</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>雷达图制作!$B$1:$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>响应快</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>体积小</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>扭力大</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>雷达图制作!$B$4:$D$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-B37B-435F-A1A5-5285699195E0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="173882544"/>
+        <c:axId val="173883984"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="173882544"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="173883984"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="173883984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="173882544"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.28782548407864111"/>
+          <c:y val="3.7845705967976713E-2"/>
+          <c:w val="0.38580779900267165"/>
+          <c:h val="4.7691427432033286E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent4"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="317">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>176212</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>100013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>133349</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="图表 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19E40572-40B7-3FA3-1CE0-D8AB9EBEB94E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1318,32 +2457,32 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1373,7 +2512,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -1389,392 +2528,387 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="49.5">
-      <c r="A2" s="5">
+      <c r="A2" s="28">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="27">
         <v>1.1574074074074073E-4</v>
       </c>
       <c r="C2" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="33">
+      <c r="A3" s="28">
+        <f t="shared" ref="A3:A9" si="0">A2+B2</f>
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="B3" s="27">
+        <v>5.7870370370370366E-5</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="29">
+        <f t="shared" si="0"/>
+        <v>1.7361111111111109E-4</v>
+      </c>
+      <c r="B4" s="30">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="33">
+      <c r="A5" s="28">
+        <f t="shared" si="0"/>
+        <v>2.8935185185185184E-4</v>
+      </c>
+      <c r="B5" s="27">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C5" s="34"/>
+      <c r="D5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="33">
-      <c r="A3" s="5">
-        <f>A2+B2</f>
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="B3" s="4">
-        <v>5.7870370370370366E-5</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="36">
-        <f>A3+B3</f>
-        <v>1.7361111111111109E-4</v>
-      </c>
-      <c r="B4" s="37">
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>125</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="E5" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="29">
+        <f t="shared" si="0"/>
+        <v>4.0509259259259258E-4</v>
+      </c>
+      <c r="B6" s="30">
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="C6" s="34"/>
+      <c r="D6" s="6" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="33">
-      <c r="A5" s="5">
-        <f>A4+B4</f>
-        <v>2.8935185185185184E-4</v>
-      </c>
-      <c r="B5" s="4">
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="36">
-        <f>A5+B5</f>
-        <v>4.0509259259259258E-4</v>
-      </c>
-      <c r="B6" s="37">
-        <v>1.1574074074074073E-5</v>
-      </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="33">
+      <c r="A7" s="28">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666664E-4</v>
+      </c>
+      <c r="B7" s="27">
+        <v>9.2592592592592588E-5</v>
+      </c>
+      <c r="C7" s="34"/>
+      <c r="D7" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="49.5">
+      <c r="A8" s="28">
+        <f t="shared" si="0"/>
+        <v>5.0925925925925921E-4</v>
+      </c>
+      <c r="B8" s="27">
+        <v>4.6296296296296294E-5</v>
+      </c>
+      <c r="C8" s="35"/>
+      <c r="D8" s="6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="33">
-      <c r="A7" s="35">
-        <f>A6+B6</f>
-        <v>4.1666666666666664E-4</v>
-      </c>
-      <c r="B7" s="34">
-        <v>9.2592592592592588E-5</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="49.5">
-      <c r="A8" s="35">
-        <f>A7+B7</f>
-        <v>5.0925925925925921E-4</v>
-      </c>
-      <c r="B8" s="34">
-        <v>4.6296296296296294E-5</v>
-      </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="6" t="s">
-        <v>37</v>
-      </c>
       <c r="E8" s="6" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="5">
-        <f>A8+B8</f>
+      <c r="A9" s="28">
+        <f t="shared" si="0"/>
         <v>5.5555555555555556E-4</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="27">
         <v>5.7870370370370366E-5</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="9" customFormat="1" ht="49.5">
-      <c r="A10" s="5">
-        <f>A8+B8</f>
+      <c r="A10" s="39">
+        <f t="shared" ref="A10:A22" si="1">A8+B8</f>
         <v>5.5555555555555556E-4</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="40">
         <v>1.3888888888888889E-4</v>
       </c>
-      <c r="C10" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>38</v>
+      <c r="C10" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>139</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="7" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="33">
-      <c r="A11" s="5">
-        <f>A9+B9</f>
+      <c r="A11" s="28">
+        <f t="shared" si="1"/>
         <v>6.134259259259259E-4</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="27">
         <v>1.3888888888888889E-4</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="6" t="s">
-        <v>60</v>
+      <c r="C11" s="34"/>
+      <c r="D11" s="41" t="s">
+        <v>135</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="11" t="s">
-        <v>113</v>
-      </c>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="33">
       <c r="A12" s="5">
-        <f>A10+B10</f>
+        <f t="shared" si="1"/>
         <v>6.9444444444444447E-4</v>
       </c>
       <c r="B12" s="4">
         <v>6.9444444444444444E-5</v>
       </c>
-      <c r="C12" s="30"/>
+      <c r="C12" s="35"/>
       <c r="D12" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F12" s="10"/>
       <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:7" s="16" customFormat="1" ht="49.5">
       <c r="A13" s="5">
-        <f>A11+B11</f>
+        <f t="shared" si="1"/>
         <v>7.5231481481481482E-4</v>
       </c>
       <c r="B13" s="4">
         <v>1.8518518518518518E-4</v>
       </c>
-      <c r="C13" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>54</v>
+      <c r="C13" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>51</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="16" customFormat="1" ht="49.5">
-      <c r="A14" s="5">
-        <f>A12+B12</f>
+      <c r="A14" s="28">
+        <f t="shared" si="1"/>
         <v>7.6388888888888893E-4</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="27">
         <v>2.3148148148148146E-4</v>
       </c>
-      <c r="C14" s="33"/>
+      <c r="C14" s="38"/>
       <c r="D14" s="14" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="F14" s="14"/>
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="16" customFormat="1" ht="115.5">
-      <c r="A15" s="5">
-        <f>A13+B13</f>
+      <c r="A15" s="28">
+        <f t="shared" si="1"/>
         <v>9.3749999999999997E-4</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="27">
         <v>3.4722222222222224E-4</v>
       </c>
-      <c r="C15" s="33"/>
+      <c r="C15" s="38"/>
       <c r="D15" s="13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
     </row>
     <row r="16" spans="1:7" s="16" customFormat="1" ht="66">
-      <c r="A16" s="5">
-        <f>A14+B14</f>
+      <c r="A16" s="28">
+        <f t="shared" si="1"/>
         <v>9.9537037037037042E-4</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="27">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C16" s="33"/>
+      <c r="C16" s="38"/>
       <c r="D16" s="13" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7" s="16" customFormat="1" ht="33">
-      <c r="A17" s="5">
-        <f>A15+B15</f>
+      <c r="A17" s="28">
+        <f t="shared" si="1"/>
         <v>1.2847222222222223E-3</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="27">
         <v>9.2592592592592588E-5</v>
       </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="13" t="s">
-        <v>41</v>
+      <c r="C17" s="38"/>
+      <c r="D17" s="32" t="s">
+        <v>38</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7" s="16" customFormat="1">
       <c r="A18" s="5">
-        <f>A16+B16</f>
+        <f t="shared" si="1"/>
         <v>1.1111111111111111E-3</v>
       </c>
       <c r="B18" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C18" s="33"/>
+      <c r="C18" s="38"/>
       <c r="D18" s="19" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E18" s="22"/>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" ht="33">
-      <c r="A19" s="5">
-        <f>A17+B17</f>
+      <c r="A19" s="39">
+        <f t="shared" si="1"/>
         <v>1.3773148148148149E-3</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="40">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="6" t="s">
-        <v>55</v>
+      <c r="C19" s="38"/>
+      <c r="D19" s="32" t="s">
+        <v>136</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
     </row>
-    <row r="20" spans="1:7" ht="66">
-      <c r="A20" s="5">
-        <f>A18+B18</f>
+    <row r="20" spans="1:7" s="47" customFormat="1" ht="66">
+      <c r="A20" s="42">
+        <f t="shared" si="1"/>
         <v>1.1226851851851851E-3</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="43">
         <v>4.0509259259259258E-4</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8" t="s">
-        <v>121</v>
+      <c r="C20" s="38"/>
+      <c r="D20" s="44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="45" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="66">
-      <c r="A21" s="5">
-        <f>A19+B19</f>
+      <c r="A21" s="39">
+        <f t="shared" si="1"/>
         <v>1.4930555555555556E-3</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="40">
         <v>2.8935185185185189E-4</v>
       </c>
-      <c r="C21" s="33"/>
-      <c r="D21" s="6" t="s">
-        <v>47</v>
+      <c r="C21" s="38"/>
+      <c r="D21" s="32" t="s">
+        <v>44</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="49.5">
-      <c r="A22" s="5">
-        <f>A20+B20</f>
+      <c r="A22" s="28">
+        <f t="shared" si="1"/>
         <v>1.5277777777777776E-3</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="27">
         <v>2.8935185185185189E-4</v>
       </c>
-      <c r="C22" s="33"/>
+      <c r="C22" s="38"/>
       <c r="D22" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="5"/>
       <c r="B23" s="4"/>
-      <c r="C23" s="33"/>
+      <c r="C23" s="38"/>
       <c r="D23" s="11" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E23" s="10"/>
     </row>
@@ -1786,197 +2920,197 @@
       <c r="B24" s="4">
         <v>1.7361111111111112E-4</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="13" t="s">
-        <v>56</v>
+      <c r="C24" s="38"/>
+      <c r="D24" s="32" t="s">
+        <v>140</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="F24" s="14"/>
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="17" customFormat="1">
       <c r="A25" s="5">
-        <f>A24+B24</f>
+        <f t="shared" ref="A25:A47" si="2">A24+B24</f>
         <v>1.9907407407407404E-3</v>
       </c>
       <c r="B25" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C25" s="33"/>
+      <c r="C25" s="38"/>
       <c r="D25" s="19" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E25" s="22"/>
       <c r="F25" s="14"/>
       <c r="G25" s="14"/>
     </row>
-    <row r="26" spans="1:7" ht="82.5">
+    <row r="26" spans="1:7" ht="66">
       <c r="A26" s="5">
-        <f>A25+B25</f>
+        <f t="shared" si="2"/>
         <v>2.0023148148148144E-3</v>
       </c>
       <c r="B26" s="4">
         <v>2.3148148148148146E-4</v>
       </c>
-      <c r="C26" s="33"/>
+      <c r="C26" s="38"/>
       <c r="D26" s="6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7" ht="99">
       <c r="A27" s="5">
-        <f>A26+B26</f>
+        <f t="shared" si="2"/>
         <v>2.2337962962962958E-3</v>
       </c>
       <c r="B27" s="4">
         <v>4.6296296296296293E-4</v>
       </c>
-      <c r="C27" s="33"/>
+      <c r="C27" s="38"/>
       <c r="D27" s="6" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="5">
-        <f>A27+B27</f>
+        <f t="shared" si="2"/>
         <v>2.6967592592592586E-3</v>
       </c>
       <c r="B28" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C28" s="33"/>
+      <c r="C28" s="38"/>
       <c r="D28" s="19" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E28" s="12"/>
     </row>
     <row r="29" spans="1:7" s="16" customFormat="1" ht="33">
       <c r="A29" s="5">
-        <f>A28+B28</f>
+        <f t="shared" si="2"/>
         <v>2.7083333333333326E-3</v>
       </c>
       <c r="B29" s="4">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C29" s="33"/>
-      <c r="D29" s="13" t="s">
-        <v>101</v>
+      <c r="C29" s="38"/>
+      <c r="D29" s="32" t="s">
+        <v>91</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="16" customFormat="1" ht="33">
       <c r="A30" s="5">
-        <f>A29+B29</f>
+        <f t="shared" si="2"/>
         <v>2.8240740740740735E-3</v>
       </c>
       <c r="B30" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C30" s="32"/>
+      <c r="C30" s="37"/>
       <c r="D30" s="13" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="19" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="5">
-        <f>A30+B30</f>
+        <f t="shared" si="2"/>
         <v>2.8819444444444439E-3</v>
       </c>
       <c r="B31" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C31" s="31" t="s">
-        <v>29</v>
+      <c r="C31" s="36" t="s">
+        <v>28</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="36">
-        <f>A31+B31</f>
+      <c r="A32" s="29">
+        <f t="shared" si="2"/>
         <v>2.9398148148148144E-3</v>
       </c>
-      <c r="B32" s="37">
+      <c r="B32" s="30">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C32" s="33"/>
+      <c r="C32" s="38"/>
       <c r="D32" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="5">
-        <f>A32+B32</f>
+        <f t="shared" si="2"/>
         <v>3.0555555555555553E-3</v>
       </c>
       <c r="B33" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C33" s="33"/>
+      <c r="C33" s="38"/>
       <c r="D33" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="33">
-      <c r="A34" s="36">
-        <f>A33+B33</f>
+      <c r="A34" s="29">
+        <f t="shared" si="2"/>
         <v>3.1134259259259257E-3</v>
       </c>
-      <c r="B34" s="37">
+      <c r="B34" s="30">
         <v>5.7870370370370378E-4</v>
       </c>
-      <c r="C34" s="33"/>
+      <c r="C34" s="38"/>
       <c r="D34" s="6" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="F34" s="7"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="36">
-        <f>A34+B34</f>
+      <c r="A35" s="29">
+        <f t="shared" si="2"/>
         <v>3.6921296296296294E-3</v>
       </c>
-      <c r="B35" s="37">
+      <c r="B35" s="30">
         <v>1.3888888888888889E-4</v>
       </c>
-      <c r="C35" s="33"/>
+      <c r="C35" s="38"/>
       <c r="D35" s="6" t="s">
         <v>7</v>
       </c>
@@ -1986,339 +3120,344 @@
       <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="36">
-        <f>A35+B35</f>
+      <c r="A36" s="29">
+        <f t="shared" si="2"/>
         <v>3.8310185185185183E-3</v>
       </c>
-      <c r="B36" s="37">
+      <c r="B36" s="30">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C36" s="33"/>
+      <c r="C36" s="38"/>
       <c r="D36" s="6" t="s">
         <v>8</v>
       </c>
       <c r="F36" s="7"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="38">
-        <f>A36+B36</f>
+      <c r="A37" s="29">
+        <f t="shared" si="2"/>
         <v>3.8888888888888888E-3</v>
       </c>
-      <c r="B37" s="39">
+      <c r="B37" s="30">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C37" s="33"/>
+      <c r="C37" s="38"/>
       <c r="D37" s="6" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="F37" s="7"/>
     </row>
     <row r="38" spans="1:7" ht="33">
-      <c r="A38" s="40">
-        <f>A37+B37</f>
+      <c r="A38" s="29">
+        <f t="shared" si="2"/>
         <v>3.9467592592592592E-3</v>
       </c>
-      <c r="B38" s="41">
+      <c r="B38" s="30">
         <v>5.7870370370370378E-4</v>
       </c>
-      <c r="C38" s="33"/>
+      <c r="C38" s="38"/>
       <c r="D38" s="6" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F38" s="7"/>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="5">
-        <f>A38+B38</f>
+        <f t="shared" si="2"/>
         <v>4.5254629629629629E-3</v>
       </c>
       <c r="B39" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C39" s="33"/>
-      <c r="D39" s="6" t="s">
+      <c r="C39" s="38"/>
+      <c r="D39" s="32" t="s">
         <v>9</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="5">
-        <f>A39+B39</f>
+        <f t="shared" si="2"/>
         <v>4.5833333333333334E-3</v>
       </c>
       <c r="B40" s="4">
         <v>3.4722222222222222E-5</v>
       </c>
-      <c r="C40" s="33"/>
-      <c r="D40" s="6" t="s">
-        <v>72</v>
+      <c r="C40" s="38"/>
+      <c r="D40" s="32" t="s">
+        <v>64</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="F40" s="7"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="5">
-        <f>A40+B40</f>
+      <c r="A41" s="28">
+        <f t="shared" si="2"/>
         <v>4.6180555555555558E-3</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="27">
         <v>4.6296296296296294E-5</v>
       </c>
-      <c r="C41" s="32"/>
+      <c r="C41" s="37"/>
       <c r="D41" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="66">
-      <c r="A42" s="5">
-        <f>A41+B41</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="33">
+      <c r="A42" s="28">
+        <f t="shared" si="2"/>
         <v>4.6643518518518518E-3</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="27">
         <v>4.6296296296296293E-4</v>
       </c>
-      <c r="C42" s="31" t="s">
-        <v>28</v>
+      <c r="C42" s="36" t="s">
+        <v>27</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>64</v>
+        <v>129</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="5">
-        <f>A42+B42</f>
+        <f t="shared" si="2"/>
         <v>5.1273148148148146E-3</v>
       </c>
       <c r="B43" s="4">
         <v>2.3148148148148147E-5</v>
       </c>
-      <c r="C43" s="33"/>
+      <c r="C43" s="38"/>
       <c r="D43" s="6" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="82.5">
       <c r="A44" s="5">
-        <f>A43+B43</f>
+        <f t="shared" si="2"/>
         <v>5.1504629629629626E-3</v>
       </c>
       <c r="B44" s="4">
         <v>4.0509259259259258E-4</v>
       </c>
-      <c r="C44" s="33"/>
+      <c r="C44" s="38"/>
       <c r="D44" s="6" t="s">
-        <v>65</v>
+        <v>132</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="5">
-        <f>A44+B44</f>
+        <f t="shared" si="2"/>
         <v>5.5555555555555549E-3</v>
       </c>
       <c r="B45" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C45" s="33"/>
+      <c r="C45" s="38"/>
       <c r="D45" s="19" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="G45" s="7"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="5"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="33"/>
-      <c r="D46" s="27" t="s">
-        <v>108</v>
+      <c r="A46" s="5">
+        <f t="shared" si="2"/>
+        <v>5.5671296296296293E-3</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C46" s="38"/>
+      <c r="D46" s="31" t="s">
+        <v>98</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G46" s="7"/>
     </row>
     <row r="47" spans="1:7" ht="66">
       <c r="A47" s="5">
-        <f>A45+B45</f>
-        <v>5.5671296296296293E-3</v>
+        <f t="shared" si="2"/>
+        <v>5.6828703703703702E-3</v>
       </c>
       <c r="B47" s="4">
         <v>4.0509259259259258E-4</v>
       </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="6" t="s">
-        <v>109</v>
+      <c r="C47" s="37"/>
+      <c r="D47" s="32" t="s">
+        <v>99</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="5">
-        <f>A47+B47</f>
-        <v>5.9722222222222216E-3</v>
+        <f t="shared" ref="A48:A56" si="3">A47+B47</f>
+        <v>6.0879629629629626E-3</v>
       </c>
       <c r="B48" s="4">
         <v>3.4722222222222222E-5</v>
       </c>
-      <c r="C48" s="31" t="s">
-        <v>27</v>
+      <c r="C48" s="36" t="s">
+        <v>26</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" s="5">
-        <f>A48+B48</f>
-        <v>6.0069444444444441E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.122685185185185E-3</v>
       </c>
       <c r="B49" s="4">
         <v>4.6296296296296294E-5</v>
       </c>
-      <c r="C49" s="33"/>
-      <c r="D49" s="6" t="s">
-        <v>19</v>
+      <c r="C49" s="38"/>
+      <c r="D49" s="32" t="s">
+        <v>18</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" s="5">
-        <f>A49+B49</f>
-        <v>6.0532407407407401E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.168981481481481E-3</v>
       </c>
       <c r="B50" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C50" s="33"/>
-      <c r="D50" s="6" t="s">
+      <c r="C50" s="38"/>
+      <c r="D50" s="32" t="s">
         <v>11</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="33">
       <c r="A51" s="5">
-        <f>A50+B50</f>
-        <v>6.1111111111111106E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.2268518518518515E-3</v>
       </c>
       <c r="B51" s="4">
         <v>6.9444444444444444E-5</v>
       </c>
-      <c r="C51" s="33"/>
-      <c r="D51" s="6" t="s">
+      <c r="C51" s="38"/>
+      <c r="D51" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" s="5">
-        <f>A51+B51</f>
-        <v>6.1805555555555546E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.2962962962962955E-3</v>
       </c>
       <c r="B52" s="4">
         <v>6.9444444444444444E-5</v>
       </c>
-      <c r="C52" s="32"/>
-      <c r="D52" s="6" t="s">
-        <v>23</v>
+      <c r="C52" s="37"/>
+      <c r="D52" s="32" t="s">
+        <v>22</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="49.5">
       <c r="A53" s="5">
-        <f>A52+B52</f>
-        <v>6.2499999999999986E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.3657407407407395E-3</v>
       </c>
       <c r="B53" s="4">
         <v>1.1574074074074073E-4</v>
       </c>
       <c r="C53" s="21"/>
       <c r="D53" s="6" t="s">
-        <v>51</v>
+        <v>142</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="33">
       <c r="A54" s="5">
-        <f>A53+B53</f>
-        <v>6.3657407407407395E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.4814814814814804E-3</v>
       </c>
       <c r="B54" s="4">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C54" s="31" t="s">
-        <v>26</v>
+      <c r="C54" s="36" t="s">
+        <v>25</v>
       </c>
       <c r="D54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F54" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="132">
       <c r="A55" s="5">
-        <f>A54+B54</f>
-        <v>6.4814814814814804E-3</v>
+        <f t="shared" si="3"/>
+        <v>6.5972222222222213E-3</v>
       </c>
       <c r="B55" s="4">
         <v>1.5046296296296294E-3</v>
       </c>
-      <c r="C55" s="32"/>
+      <c r="C55" s="37"/>
       <c r="D55" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" s="5">
-        <f>A55+B55</f>
-        <v>7.9861111111111105E-3</v>
+        <f t="shared" si="3"/>
+        <v>8.1018518518518514E-3</v>
       </c>
       <c r="C56" s="25" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2337,16 +3476,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{543450A5-C08D-4873-BAC4-1F306BA55BCC}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14"/>
-  <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F25715-BEED-42F5-8F10-9FEA1FF7F5C3}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14"/>
@@ -2357,16 +3486,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2374,10 +3503,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2385,10 +3514,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2396,14 +3525,82 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5D1F29C-200F-4BB5-9251-208FEB1786B7}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="10.58203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>6</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1: Update the screenplay. prototype: No model has been updated, Only generate an exploded view for animation.
</commit_message>
<xml_diff>
--- a/v1/screenplay_zh.xlsx
+++ b/v1/screenplay_zh.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEV\project\self_playing_ruler\v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B928CA9-3714-458F-9477-6C58C5B77891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4D9E5B-5BC9-4182-838F-078339DDD8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-130" yWindow="-130" windowWidth="25860" windowHeight="13940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="封标" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="138">
   <si>
     <t>​​画面描述 (分镜)​​</t>
   </si>
@@ -62,9 +62,6 @@
     <t>响指</t>
   </si>
   <si>
-    <t>重新建模，将主板与钢尺、电机等整合在一起</t>
-  </si>
-  <si>
     <t>模型爆炸图</t>
   </si>
   <si>
@@ -77,18 +74,11 @@
     <t>主要模块的代码展示</t>
   </si>
   <si>
-    <t>笔吹奏演示</t>
-  </si>
-  <si>
     <t xml:space="preserve">​​时间戳 </t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>在屏幕前打一个响指，PCB出现在桌面</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>按照新的设计，开干！！！</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -105,31 +95,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>拨动钢尺演奏示意</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>这是管乐</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>pen beats演示（两次动次打次）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>第二遍跟读：动次打次
-这是打击乐</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>贝斯（钢尺），长笛（笔），架子鼓（笔）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1个钢尺琴--&gt;2个钢尺琴--&gt;3个钢尺琴</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>气泡音</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -159,14 +124,6 @@
   </si>
   <si>
     <t>片头</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>手动演奏一个《小星星》</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>早年在b站看大佬用钢尺演奏太酷了！我也要！</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -188,10 +145,6 @@
   <si>
     <t>当前滑块特写
 光驱内部结构特写</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>连线图待绘制</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -252,26 +205,11 @@
   </si>
   <si>
     <t>口播出镜
-慢速演奏（正常）
-快速（无法压住钢尺，节奏乱掉）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>口播出镜
 展示一个串口谱子</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>连线图
-外面一个框浮现</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>演奏前：来看看效果吧！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>接下来就要注入灵魂，撸代码！！！</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -299,14 +237,6 @@
     <t>口播出镜</t>
   </si>
   <si>
-    <t>不过一只钢尺演奏难免有些单调，所以我希望在增加几个乐器</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>怎么样？这个赛博钢尺琴是不是还有点意思？</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>赛 博 钢 尺 琴——DIY自动演奏的钢尺</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -323,26 +253,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>夺舍BGM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>最后的最后，虽然只有一种乐器，也可以用多个组多声部
-接下来就以一首《卡农》作为结尾</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>一个转场动画</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>钢琴一个八度的排列，12个音
-切换到特写键盘do与升do
-指示&lt;50音分偏差
-指示&gt;50音分偏差</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>原理图--&gt;pcb--&gt;2D渲染图</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -352,10 +266,6 @@
   </si>
   <si>
     <t>结束</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>再加上钢尺作为贝斯，让它们组一个文具乐队！！！</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -374,10 +284,6 @@
   </si>
   <si>
     <t>《spoiler》</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>钢尺君演奏片段</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -416,29 +322,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>解决了速度问题，下一个要解决的就是音不准的问题
-偏差有x.x%，如果偏差超过3%（50音分）就是明显跑调了</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>这是因为我们常见的音乐都是使用十二平均律，将一个八度平均分成十二份,一份就是一个半音，一个半音音程等于100音分。假设我弹奏一个do，如果偏差小于50音分，它更接近do，可能有些不准但还可以听出来是do。但如果偏差超过50音分，那它就更接近升do了，也就是跑调了。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>如何提高音准呢？
-此前调音是在桌面拨动钢尺，用手机测出几个基准长度的音高，而后拟合出频率-长度函数。演奏的时候通过目标频率换算出具体长度。但这样人工测量非常耗时，而且并不准确</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>因此，需要添加一个麦克风，在不同长度的位置拨动钢尺，用麦克风采集音频并进行傅里叶变换，得到对应长度的频率。最终就可以拟合出一个高精度的频率-步进(step)曲线</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>既然为了调音增加了麦克风硬件，那为什么不物尽其用呢？
-esp32s3开发板刚好有usb接口，可以集成一个usb麦克风，连接电脑用来录音，获得更好的录音音质。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>10:19-10:32 https://www.bilibili.com/video/BV187411r7hp/</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -451,27 +334,8 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>哎！不知道你有没有听过一种技术叫MIDI，它即可以传输音符，又可以存储乐谱。
-功能机时代的诺基亚铃声，你一定听过
-它就是midi
-midi可以使用多种接口进行传输，比如usb接口。而刚好我们的开发板上就有usb接口。使用usb midi就是最好的选择了。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>开发板乱糟糟的连线
 人+影视飓风的扭转特效</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>最后，使用面包板，各种连线实在太乱了</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>画一个电路板，把它们整合起来</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>为了更方便复刻，都是使用的成品模块</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -499,16 +363,8 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>（可以先用记号笔标注一下钢尺上音的位置）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>先试试最简单的小星星
 这是《小星星》？我自己都要听不出来了？</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>TODO：这里应该对比人手弹奏时的动作</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -554,10 +410,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>TODO：需要实测一下瀑布图，看看频率变化</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>我：那怎么办呢？
 刘华强：那，吸铁石
 我：对呀！谁说一定要用舵机呢。钢尺嘛，可以用电磁铁来吸住它
@@ -571,10 +423,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>TODO:删除</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>引子</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -651,37 +499,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>演奏《小星星》</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">夺舍（使用伤心欲茄声音AI合成）：斯你麻赛，nice什么呀！修改了多少个版本才有现在的效果的呀？你是nice了，我的刻度线都磨没了，八嘎压路！
-我：这不是考虑到观众老爷的观看体验，将中间的调试过程压缩了么
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>我：结构上迭代设计了很多版，看，盒子里有好多
-我：代码也是改了很多次，这里有100多个commit</t>
-    </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -726,24 +544,17 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>口播出镜
-自动弹奏一个音+手机fft，浮现文字：误差xxx</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>演奏一个音符的慢放视频（使用类似进度条的东西，显示每部分时间占用）</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>我先设计了一个原型机验证可行性
-模仿演奏的动作，使用丝杆步进电机来精确控制钢尺移动、
-使用一个舵机压住钢尺、另一个舵机弹拨钢尺</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>手绘设计图展示</t>
-    </r>
+    <t>还有一个问题，就是，乐谱的存储与传输
+原型机的谱子格式是自定义的：
+比如，("5", 1)：即表示Sol，时长为一拍，用串口发送一个音符演奏一个音符
+这样，虽然调试方便，但每首歌都要一个音一个音来写，太麻烦了！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -753,7 +564,7 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>（舵机、丝杆步进电机）</t>
+      <t>插入电脑</t>
     </r>
     <r>
       <rPr>
@@ -764,25 +575,221 @@
         <charset val="134"/>
       </rPr>
       <t xml:space="preserve">
-每个器件特写气泡（根据口播节奏依次出现）</t>
+设备管理器与音频设备展示</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>最后的最后，就以一首《卡农》二重奏作为结尾吧</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>口播出镜
-麦克风--&gt;开发板-(usb线)-&gt;mic--电脑
-添加一个DRI Mic的在音频设备中的截图</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>还有一个问题，就是，乐谱的存储与传输
-原型机的谱子格式是自定义的：
-比如，("5", 1)：即表示Sol，时长为一拍，用串口发送一个音符演奏一个音符
-这样，虽然调试方便，但每首歌都要一个音一个音来写，太麻烦了！！！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>；</t>
+快速演奏（无法压住钢尺，节奏乱掉）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">口播出镜
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-0.14999847407452621"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>自动弹奏一个音+手机fft，浮现文字：误差xxx</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">解决了速度问题，下一个要解决的就是音不准的问题
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-0.14999847407452621"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>偏差有x.x%，如果偏差超过3%（50音分）就是明显跑调了</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>因此，使用程序控制钢尺在不同长度弹奏，并用麦克风采集音频进行傅里叶变换，得到对应长度的频率。最终就可以拟合出一个高精度的频率-电机步进(step)曲线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+麦克风--&gt;开发板-(usb线)-&gt;mic--电脑</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>既然有了麦克风硬件和usb，那为什么不物尽其用呢？
+可以再集成一个usb麦克风，连接电脑用来录音，获得更好的录音音质。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>哎！不知道你有没有听过一种技术叫MIDI，它即可以传输音符，又可以存储乐谱。
+举个例子，功能机时代的诺基亚铃声，它就是midi
+midi可以使用多种接口进行传输，比如usb接口。而esp32主控就支持usb接口。使用usb midi就是最好的选择了。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>如何提高音准呢？先看一下原型机上的方法：
+调音时，在桌面拨动钢尺，用手机测出几个基准长度的音高，而后拟合出频率-长度函数。
+演奏的，时候通过目标频率换算出具体长度。
+但这样人工测量非常耗时，而且并不准确。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>那么，开干！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>最后，使用开发板+面包板飞线，实在太乱了。
+需要一个新设计把他们整合起来！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+做出握拳加油的手势</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TODO：做一下视频增稳</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>怎么样？这个赛博钢尺琴是不是还有点意思？
+不过单单一只钢尺演奏难免有些单调，所以我希望再增加几个乐器</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>首先是钢尺，充当类似吉他的角色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>其次是第一支笔，充当类似长笛的角色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>pen beats演示动次打次三次（缩小并放在右下角，配架子鼓）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>拨动钢尺演奏示意（缩小并放在左下角，配吉他）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>吹笔奏演示意（缩小并放在上方，配长笛）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>第二开始遍跟读：动次打次
+这是第二支笔，充当类似架子鼓的角色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>让它们组一个文具乐队！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>吉他（钢尺），长笛（笔），架子鼓（笔）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>首先设计一个原型机，验证可行性。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>加入一下飞入的音效</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>先画一个个手绘示意图
+然后来建模，使用丝杆步进电机来控制钢尺移动、使用一个舵机压住钢尺、另一个舵机弹拨钢尺。最后加上底座就完成啦！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>早年在b站经常能看到大佬用钢尺演奏音乐，比如这个
+（视频播放）
+真是太酷了！我也跃跃欲试，想要自己演奏试试！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播
+千本樱——佚名
+only my railgun——钢尺君
+大东北我的家乡——杯鸽
+（以相片的方式一次落下堆叠）
+口播</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播
+手动演奏一个《小星星》</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TODO:文本霓虹灯特效</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>手绘设计图展示
+建模展示：钢尺+丝杆步进电机+按压舵机+拨弦舵机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>首先设计PCB，为了更方便复刻，都是使用的成品模块</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>重新建模，将主板与钢尺、电机等器件整合在一起</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>搞定了硬件，接下来就要注入灵魂，撸代码！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>leonierX</t>
+  </si>
+  <si>
+    <t>nokia tune (MIDI)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">夺舍（使用伤心欲茄声音AI合成）：斯你麻赛，nice什么呀！修改了多少个版本才有现在的效果的呀？你是nice了，我的刻度线都磨没了，八嘎压路！
+我：这不是考虑到观众老爷的观看体验，将中间的调试过程压缩了么
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>我：当然，制作过程还是有些波折的。看，盒子里都是结构建模迭代的版本。
+我：代码也是改了很多次，这里有100多个commit</t>
+    </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -790,7 +797,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="等线"/>
@@ -859,6 +866,13 @@
     <font>
       <sz val="11"/>
       <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.14999847407452621"/>
       <name val="微软雅黑"/>
       <family val="2"/>
       <charset val="134"/>
@@ -998,7 +1012,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1092,15 +1106,24 @@
     <xf numFmtId="45" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="21" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="21" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="21" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="21" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1116,13 +1139,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="21" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="21" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1132,12 +1149,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2457,32 +2468,32 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="20" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="20" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2493,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultColWidth="9.08203125" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="2" width="8.25" style="6" customWidth="1"/>
@@ -2506,13 +2517,13 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -2528,41 +2539,44 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="49.5">
-      <c r="A2" s="28">
+      <c r="A2" s="29">
         <v>0</v>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="30">
         <v>1.1574074074074073E-4</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="33">
-      <c r="A3" s="28">
+      <c r="A3" s="29">
         <f t="shared" ref="A3:A9" si="0">A2+B2</f>
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="30">
         <v>5.7870370370370366E-5</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>134</v>
+        <v>97</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>57</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="99">
       <c r="A4" s="29">
         <f t="shared" si="0"/>
         <v>1.7361111111111109E-4</v>
@@ -2570,14 +2584,14 @@
       <c r="B4" s="30">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C4" s="33" t="s">
-        <v>110</v>
+      <c r="C4" s="36" t="s">
+        <v>75</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>79</v>
+        <v>128</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>33</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="33">
@@ -2588,15 +2602,12 @@
       <c r="B5" s="27">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C5" s="34"/>
+      <c r="C5" s="37"/>
       <c r="D5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="41" t="s">
-        <v>101</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>100</v>
+        <v>129</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -2607,13 +2618,13 @@
       <c r="B6" s="30">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="37"/>
       <c r="D6" s="6" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="33">
@@ -2624,12 +2635,12 @@
       <c r="B7" s="27">
         <v>9.2592592592592588E-5</v>
       </c>
-      <c r="C7" s="34"/>
+      <c r="C7" s="37"/>
       <c r="D7" s="26" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>133</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="49.5">
@@ -2640,12 +2651,12 @@
       <c r="B8" s="27">
         <v>4.6296296296296294E-5</v>
       </c>
-      <c r="C8" s="35"/>
+      <c r="C8" s="38"/>
       <c r="D8" s="6" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2657,818 +2668,799 @@
         <v>5.7870370370370366E-5</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="9" customFormat="1" ht="49.5">
-      <c r="A10" s="39">
-        <f t="shared" ref="A10:A22" si="1">A8+B8</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="9" customFormat="1">
+      <c r="A10" s="32">
+        <f>A7+B7</f>
+        <v>5.0925925925925921E-4</v>
+      </c>
+      <c r="B10" s="33">
+        <v>1.3888888888888889E-4</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:7" s="9" customFormat="1" ht="49.5">
+      <c r="A11" s="32">
+        <f>A8+B8</f>
         <v>5.5555555555555556E-4</v>
       </c>
-      <c r="B10" s="40">
+      <c r="B11" s="33">
         <v>1.3888888888888889E-4</v>
       </c>
-      <c r="C10" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="33">
-      <c r="A11" s="28">
-        <f t="shared" si="1"/>
+      <c r="C11" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" ht="33">
+      <c r="A12" s="28">
+        <f>A9+B9</f>
         <v>6.134259259259259E-4</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B12" s="27">
         <v>1.3888888888888889E-4</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="41" t="s">
-        <v>135</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="11"/>
-    </row>
-    <row r="12" spans="1:7" ht="33">
-      <c r="A12" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9444444444444447E-4</v>
-      </c>
-      <c r="B12" s="4">
-        <v>6.9444444444444444E-5</v>
-      </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>81</v>
+      <c r="C12" s="37"/>
+      <c r="D12" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="F12" s="10"/>
       <c r="G12" s="11"/>
     </row>
-    <row r="13" spans="1:7" s="16" customFormat="1" ht="49.5">
+    <row r="13" spans="1:7" ht="33">
       <c r="A13" s="5">
-        <f t="shared" si="1"/>
-        <v>7.5231481481481482E-4</v>
+        <f t="shared" ref="A13:A20" si="1">A11+B11</f>
+        <v>6.9444444444444447E-4</v>
       </c>
       <c r="B13" s="4">
-        <v>1.8518518518518518E-4</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="G13" s="14"/>
+        <v>6.9444444444444444E-5</v>
+      </c>
+      <c r="C13" s="38"/>
+      <c r="D13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="10"/>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" spans="1:7" s="16" customFormat="1" ht="49.5">
       <c r="A14" s="28">
         <f t="shared" si="1"/>
-        <v>7.6388888888888893E-4</v>
+        <v>7.5231481481481482E-4</v>
       </c>
       <c r="B14" s="27">
-        <v>2.3148148148148146E-4</v>
-      </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="F14" s="14"/>
+        <v>1.8518518518518518E-4</v>
+      </c>
+      <c r="C14" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>94</v>
+      </c>
       <c r="G14" s="14"/>
     </row>
-    <row r="15" spans="1:7" s="16" customFormat="1" ht="115.5">
+    <row r="15" spans="1:7" s="16" customFormat="1" ht="49.5">
       <c r="A15" s="28">
         <f t="shared" si="1"/>
-        <v>9.3749999999999997E-4</v>
+        <v>7.6388888888888893E-4</v>
       </c>
       <c r="B15" s="27">
-        <v>3.4722222222222224E-4</v>
-      </c>
-      <c r="C15" s="38"/>
-      <c r="D15" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="1:7" s="16" customFormat="1" ht="66">
+        <v>2.3148148148148146E-4</v>
+      </c>
+      <c r="C15" s="41"/>
+      <c r="D15" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="14"/>
+      <c r="G15" s="19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="16" customFormat="1" ht="115.5">
       <c r="A16" s="28">
         <f t="shared" si="1"/>
-        <v>9.9537037037037042E-4</v>
+        <v>9.3749999999999997E-4</v>
       </c>
       <c r="B16" s="27">
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="C16" s="38"/>
+        <v>3.4722222222222224E-4</v>
+      </c>
+      <c r="C16" s="41"/>
       <c r="D16" s="13" t="s">
-        <v>108</v>
+        <v>37</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>37</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="F16" s="13"/>
       <c r="G16" s="13"/>
     </row>
-    <row r="17" spans="1:7" s="16" customFormat="1" ht="33">
+    <row r="17" spans="1:7" s="16" customFormat="1" ht="66">
       <c r="A17" s="28">
         <f t="shared" si="1"/>
+        <v>9.9537037037037042E-4</v>
+      </c>
+      <c r="B17" s="27">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C17" s="41"/>
+      <c r="D17" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="1:7" s="16" customFormat="1" ht="33">
+      <c r="A18" s="28">
+        <f t="shared" si="1"/>
         <v>1.2847222222222223E-3</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B18" s="27">
         <v>9.2592592592592588E-5</v>
       </c>
-      <c r="C17" s="38"/>
-      <c r="D17" s="32" t="s">
+      <c r="C18" s="41"/>
+      <c r="D18" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-    </row>
-    <row r="18" spans="1:7" s="16" customFormat="1">
-      <c r="A18" s="5">
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="1:7" s="16" customFormat="1">
+      <c r="A19" s="5">
         <f t="shared" si="1"/>
         <v>1.1111111111111111E-3</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B19" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-    </row>
-    <row r="19" spans="1:7" ht="33">
-      <c r="A19" s="39">
+      <c r="C19" s="41"/>
+      <c r="D19" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="22"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" spans="1:7" ht="33">
+      <c r="A20" s="32">
         <f t="shared" si="1"/>
         <v>1.3773148148148149E-3</v>
       </c>
-      <c r="B19" s="40">
+      <c r="B20" s="33">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C19" s="38"/>
-      <c r="D19" s="32" t="s">
-        <v>136</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-    </row>
-    <row r="20" spans="1:7" s="47" customFormat="1" ht="66">
-      <c r="A20" s="42">
-        <f t="shared" si="1"/>
-        <v>1.1226851851851851E-3</v>
-      </c>
-      <c r="B20" s="43">
-        <v>4.0509259259259258E-4</v>
-      </c>
-      <c r="C20" s="38"/>
-      <c r="D20" s="44" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="66">
-      <c r="A21" s="39">
-        <f t="shared" si="1"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+    </row>
+    <row r="21" spans="1:7" ht="82.5">
+      <c r="A21" s="28">
+        <f>A20+B20</f>
         <v>1.4930555555555556E-3</v>
       </c>
-      <c r="B21" s="40">
+      <c r="B21" s="27">
         <v>2.8935185185185189E-4</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="32" t="s">
-        <v>44</v>
+      <c r="C21" s="41"/>
+      <c r="D21" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="49.5">
       <c r="A22" s="28">
-        <f t="shared" si="1"/>
-        <v>1.5277777777777776E-3</v>
+        <f>A21+B21</f>
+        <v>1.7824074074074075E-3</v>
       </c>
       <c r="B22" s="27">
         <v>2.8935185185185189E-4</v>
       </c>
-      <c r="C22" s="38"/>
+      <c r="C22" s="41"/>
       <c r="D22" s="10" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="5"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="38"/>
+      <c r="A23" s="32">
+        <f t="shared" ref="A23:A24" si="2">A22+B22</f>
+        <v>2.0717592592592593E-3</v>
+      </c>
+      <c r="B23" s="33">
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="C23" s="41"/>
       <c r="D23" s="11" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="E23" s="10"/>
     </row>
-    <row r="24" spans="1:7" s="17" customFormat="1" ht="49.5">
-      <c r="A24" s="5">
-        <f>A22+B22</f>
-        <v>1.8171296296296295E-3</v>
-      </c>
-      <c r="B24" s="4">
+    <row r="24" spans="1:7" ht="66">
+      <c r="A24" s="28">
+        <f t="shared" si="2"/>
+        <v>2.0833333333333333E-3</v>
+      </c>
+      <c r="B24" s="27">
+        <v>2.3148148148148146E-4</v>
+      </c>
+      <c r="C24" s="41"/>
+      <c r="D24" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" spans="1:7" ht="82.5">
+      <c r="A25" s="28">
+        <f t="shared" ref="A25:A46" si="3">A24+B24</f>
+        <v>2.3148148148148147E-3</v>
+      </c>
+      <c r="B25" s="27">
+        <v>4.6296296296296293E-4</v>
+      </c>
+      <c r="C25" s="41"/>
+      <c r="D25" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="5">
+        <f>A25+B25</f>
+        <v>2.7777777777777775E-3</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="C26" s="41"/>
+      <c r="D26" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="12"/>
+    </row>
+    <row r="27" spans="1:7" s="17" customFormat="1" ht="33">
+      <c r="A27" s="28">
+        <f>A26+B26</f>
+        <v>2.7893518518518515E-3</v>
+      </c>
+      <c r="B27" s="27">
         <v>1.7361111111111112E-4</v>
       </c>
-      <c r="C24" s="38"/>
-      <c r="D24" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-    </row>
-    <row r="25" spans="1:7" s="17" customFormat="1">
-      <c r="A25" s="5">
-        <f t="shared" ref="A25:A47" si="2">A24+B24</f>
-        <v>1.9907407407407404E-3</v>
-      </c>
-      <c r="B25" s="4">
-        <v>1.1574074074074073E-5</v>
-      </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E25" s="22"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-    </row>
-    <row r="26" spans="1:7" ht="66">
-      <c r="A26" s="5">
-        <f t="shared" si="2"/>
-        <v>2.0023148148148144E-3</v>
-      </c>
-      <c r="B26" s="4">
-        <v>2.3148148148148146E-4</v>
-      </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-    </row>
-    <row r="27" spans="1:7" ht="99">
-      <c r="A27" s="5">
-        <f t="shared" si="2"/>
-        <v>2.2337962962962958E-3</v>
-      </c>
-      <c r="B27" s="4">
-        <v>4.6296296296296293E-4</v>
-      </c>
-      <c r="C27" s="38"/>
-      <c r="D27" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="C27" s="41"/>
+      <c r="D27" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+    </row>
+    <row r="28" spans="1:7" s="17" customFormat="1">
       <c r="A28" s="5">
-        <f t="shared" si="2"/>
-        <v>2.6967592592592586E-3</v>
+        <f>A27+B27</f>
+        <v>2.9629629629629624E-3</v>
       </c>
       <c r="B28" s="4">
         <v>1.1574074074074073E-5</v>
       </c>
-      <c r="C28" s="38"/>
+      <c r="C28" s="41"/>
       <c r="D28" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E28" s="12"/>
+        <v>50</v>
+      </c>
+      <c r="E28" s="22"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" s="16" customFormat="1" ht="33">
-      <c r="A29" s="5">
-        <f t="shared" si="2"/>
-        <v>2.7083333333333326E-3</v>
-      </c>
-      <c r="B29" s="4">
+      <c r="A29" s="28">
+        <f>A28+B28</f>
+        <v>2.9745370370370364E-3</v>
+      </c>
+      <c r="B29" s="27">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C29" s="38"/>
-      <c r="D29" s="32" t="s">
-        <v>91</v>
+      <c r="C29" s="41"/>
+      <c r="D29" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
     </row>
-    <row r="30" spans="1:7" s="16" customFormat="1" ht="33">
-      <c r="A30" s="5">
-        <f t="shared" si="2"/>
-        <v>2.8240740740740735E-3</v>
+    <row r="30" spans="1:7">
+      <c r="A30" s="32">
+        <f>A29+B29</f>
+        <v>3.0902777777777773E-3</v>
       </c>
       <c r="B30" s="4">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C30" s="37"/>
-      <c r="D30" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F30" s="13"/>
-      <c r="G30" s="19" t="s">
-        <v>39</v>
+      <c r="C30" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="5">
-        <f t="shared" si="2"/>
-        <v>2.8819444444444439E-3</v>
-      </c>
-      <c r="B31" s="4">
+      <c r="A31" s="29">
+        <f t="shared" si="3"/>
+        <v>3.1481481481481477E-3</v>
+      </c>
+      <c r="B31" s="30">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C31" s="41"/>
+      <c r="D31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="46" customFormat="1">
+      <c r="A32" s="43">
+        <f t="shared" si="3"/>
+        <v>3.2638888888888887E-3</v>
+      </c>
+      <c r="B32" s="44">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C31" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="29">
-        <f t="shared" si="2"/>
-        <v>2.9398148148148144E-3</v>
-      </c>
-      <c r="B32" s="30">
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="C32" s="38"/>
-      <c r="D32" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" s="5">
-        <f t="shared" si="2"/>
-        <v>3.0555555555555553E-3</v>
-      </c>
-      <c r="B33" s="4">
-        <v>5.7870370370370366E-5</v>
-      </c>
-      <c r="C33" s="38"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="45" t="s">
+        <v>52</v>
+      </c>
+      <c r="F32" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" s="45"/>
+    </row>
+    <row r="33" spans="1:7" ht="33">
+      <c r="A33" s="29">
+        <f t="shared" si="3"/>
+        <v>3.3217592592592591E-3</v>
+      </c>
+      <c r="B33" s="30">
+        <v>5.7870370370370378E-4</v>
+      </c>
+      <c r="C33" s="41"/>
       <c r="D33" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="33">
+        <v>64</v>
+      </c>
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" s="29">
-        <f t="shared" si="2"/>
-        <v>3.1134259259259257E-3</v>
+        <f t="shared" si="3"/>
+        <v>3.9004629629629628E-3</v>
       </c>
       <c r="B34" s="30">
-        <v>5.7870370370370378E-4</v>
-      </c>
-      <c r="C34" s="38"/>
+        <v>1.3888888888888889E-4</v>
+      </c>
+      <c r="C34" s="41"/>
       <c r="D34" s="6" t="s">
-        <v>95</v>
+        <v>6</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>133</v>
       </c>
       <c r="F34" s="7"/>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="29">
-        <f t="shared" si="2"/>
-        <v>3.6921296296296294E-3</v>
+        <f t="shared" si="3"/>
+        <v>4.0393518518518513E-3</v>
       </c>
       <c r="B35" s="30">
-        <v>1.3888888888888889E-4</v>
-      </c>
-      <c r="C35" s="38"/>
+        <v>5.7870370370370366E-5</v>
+      </c>
+      <c r="C35" s="41"/>
       <c r="D35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>6</v>
-      </c>
       <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="29">
-        <f t="shared" si="2"/>
-        <v>3.8310185185185183E-3</v>
+        <f t="shared" si="3"/>
+        <v>4.0972222222222217E-3</v>
       </c>
       <c r="B36" s="30">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C36" s="38"/>
+      <c r="C36" s="41"/>
       <c r="D36" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37" spans="1:7" ht="33">
+      <c r="A37" s="29">
+        <f t="shared" si="3"/>
+        <v>4.1550925925925922E-3</v>
+      </c>
+      <c r="B37" s="30">
+        <v>5.7870370370370378E-4</v>
+      </c>
+      <c r="C37" s="41"/>
+      <c r="D37" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F37" s="7"/>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="29">
+        <f t="shared" si="3"/>
+        <v>4.7337962962962958E-3</v>
+      </c>
+      <c r="B38" s="30">
+        <v>5.7870370370370366E-5</v>
+      </c>
+      <c r="C38" s="41"/>
+      <c r="D38" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="F36" s="7"/>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="29">
-        <f t="shared" si="2"/>
-        <v>3.8888888888888888E-3</v>
-      </c>
-      <c r="B37" s="30">
+      <c r="F38" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="28">
+        <f t="shared" si="3"/>
+        <v>4.7916666666666663E-3</v>
+      </c>
+      <c r="B39" s="27">
+        <v>3.4722222222222222E-5</v>
+      </c>
+      <c r="C39" s="41"/>
+      <c r="D39" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="28">
+        <f t="shared" si="3"/>
+        <v>4.8263888888888887E-3</v>
+      </c>
+      <c r="B40" s="27">
+        <v>4.6296296296296294E-5</v>
+      </c>
+      <c r="C40" s="40"/>
+      <c r="D40" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="33">
+      <c r="A41" s="32">
+        <f t="shared" si="3"/>
+        <v>4.8726851851851848E-3</v>
+      </c>
+      <c r="B41" s="33">
+        <v>4.6296296296296293E-4</v>
+      </c>
+      <c r="C41" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="28">
+        <f t="shared" si="3"/>
+        <v>5.3356481481481475E-3</v>
+      </c>
+      <c r="B42" s="27">
+        <v>2.3148148148148147E-5</v>
+      </c>
+      <c r="C42" s="41"/>
+      <c r="D42" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="99">
+      <c r="A43" s="28">
+        <f t="shared" si="3"/>
+        <v>5.3587962962962955E-3</v>
+      </c>
+      <c r="B43" s="27">
+        <v>4.0509259259259258E-4</v>
+      </c>
+      <c r="C43" s="41"/>
+      <c r="D43" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="5">
+        <f t="shared" si="3"/>
+        <v>5.7638888888888878E-3</v>
+      </c>
+      <c r="B44" s="4">
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="C44" s="41"/>
+      <c r="D44" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="G44" s="7"/>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="28">
+        <f t="shared" si="3"/>
+        <v>5.7754629629629623E-3</v>
+      </c>
+      <c r="B45" s="27">
+        <v>1.1574074074074073E-4</v>
+      </c>
+      <c r="C45" s="41"/>
+      <c r="D45" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G45" s="7"/>
+    </row>
+    <row r="46" spans="1:7" ht="66">
+      <c r="A46" s="28">
+        <f t="shared" si="3"/>
+        <v>5.8912037037037032E-3</v>
+      </c>
+      <c r="B46" s="27">
+        <v>4.0509259259259258E-4</v>
+      </c>
+      <c r="C46" s="40"/>
+      <c r="D46" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="33">
+      <c r="A47" s="5">
+        <f t="shared" ref="A47:A55" si="4">A46+B46</f>
+        <v>6.2962962962962955E-3</v>
+      </c>
+      <c r="B47" s="4">
+        <v>3.4722222222222222E-5</v>
+      </c>
+      <c r="C47" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="28">
+        <f t="shared" si="4"/>
+        <v>6.3310185185185179E-3</v>
+      </c>
+      <c r="B48" s="27">
+        <v>4.6296296296296294E-5</v>
+      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="28">
+        <f t="shared" si="4"/>
+        <v>6.377314814814814E-3</v>
+      </c>
+      <c r="B49" s="27">
         <v>5.7870370370370366E-5</v>
       </c>
-      <c r="C37" s="38"/>
-      <c r="D37" s="6" t="s">
+      <c r="C49" s="41"/>
+      <c r="D49" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="33">
+      <c r="A50" s="28">
+        <f t="shared" si="4"/>
+        <v>6.4351851851851844E-3</v>
+      </c>
+      <c r="B50" s="27">
+        <v>6.9444444444444444E-5</v>
+      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="28">
+        <f t="shared" si="4"/>
+        <v>6.5046296296296284E-3</v>
+      </c>
+      <c r="B51" s="27">
+        <v>6.9444444444444444E-5</v>
+      </c>
+      <c r="C51" s="40"/>
+      <c r="D51" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="F37" s="7"/>
-    </row>
-    <row r="38" spans="1:7" ht="33">
-      <c r="A38" s="29">
-        <f t="shared" si="2"/>
-        <v>3.9467592592592592E-3</v>
-      </c>
-      <c r="B38" s="30">
-        <v>5.7870370370370378E-4</v>
-      </c>
-      <c r="C38" s="38"/>
-      <c r="D38" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="F38" s="7"/>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="5">
-        <f t="shared" si="2"/>
-        <v>4.5254629629629629E-3</v>
-      </c>
-      <c r="B39" s="4">
-        <v>5.7870370370370366E-5</v>
-      </c>
-      <c r="C39" s="38"/>
-      <c r="D39" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="5">
-        <f t="shared" si="2"/>
-        <v>4.5833333333333334E-3</v>
-      </c>
-      <c r="B40" s="4">
-        <v>3.4722222222222222E-5</v>
-      </c>
-      <c r="C40" s="38"/>
-      <c r="D40" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F40" s="7"/>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="28">
-        <f t="shared" si="2"/>
-        <v>4.6180555555555558E-3</v>
-      </c>
-      <c r="B41" s="27">
-        <v>4.6296296296296294E-5</v>
-      </c>
-      <c r="C41" s="37"/>
-      <c r="D41" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="33">
-      <c r="A42" s="28">
-        <f t="shared" si="2"/>
-        <v>4.6643518518518518E-3</v>
-      </c>
-      <c r="B42" s="27">
-        <v>4.6296296296296293E-4</v>
-      </c>
-      <c r="C42" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" s="5">
-        <f t="shared" si="2"/>
-        <v>5.1273148148148146E-3</v>
-      </c>
-      <c r="B43" s="4">
-        <v>2.3148148148148147E-5</v>
-      </c>
-      <c r="C43" s="38"/>
-      <c r="D43" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="82.5">
-      <c r="A44" s="5">
-        <f t="shared" si="2"/>
-        <v>5.1504629629629626E-3</v>
-      </c>
-      <c r="B44" s="4">
-        <v>4.0509259259259258E-4</v>
-      </c>
-      <c r="C44" s="38"/>
-      <c r="D44" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" s="5">
-        <f t="shared" si="2"/>
-        <v>5.5555555555555549E-3</v>
-      </c>
-      <c r="B45" s="4">
-        <v>1.1574074074074073E-5</v>
-      </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G45" s="7"/>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" s="5">
-        <f t="shared" si="2"/>
-        <v>5.5671296296296293E-3</v>
-      </c>
-      <c r="B46" s="4">
+    </row>
+    <row r="52" spans="1:7" ht="49.5">
+      <c r="A52" s="5">
+        <f t="shared" si="4"/>
+        <v>6.5740740740740725E-3</v>
+      </c>
+      <c r="B52" s="4">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C46" s="38"/>
-      <c r="D46" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="G46" s="7"/>
-    </row>
-    <row r="47" spans="1:7" ht="66">
-      <c r="A47" s="5">
-        <f t="shared" si="2"/>
-        <v>5.6828703703703702E-3</v>
-      </c>
-      <c r="B47" s="4">
-        <v>4.0509259259259258E-4</v>
-      </c>
-      <c r="C47" s="37"/>
-      <c r="D47" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
-      <c r="A48" s="5">
-        <f t="shared" ref="A48:A56" si="3">A47+B47</f>
-        <v>6.0879629629629626E-3</v>
-      </c>
-      <c r="B48" s="4">
-        <v>3.4722222222222222E-5</v>
-      </c>
-      <c r="C48" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" s="5">
-        <f t="shared" si="3"/>
-        <v>6.122685185185185E-3</v>
-      </c>
-      <c r="B49" s="4">
-        <v>4.6296296296296294E-5</v>
-      </c>
-      <c r="C49" s="38"/>
-      <c r="D49" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="5">
-        <f t="shared" si="3"/>
-        <v>6.168981481481481E-3</v>
-      </c>
-      <c r="B50" s="4">
-        <v>5.7870370370370366E-5</v>
-      </c>
-      <c r="C50" s="38"/>
-      <c r="D50" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="33">
-      <c r="A51" s="5">
-        <f t="shared" si="3"/>
-        <v>6.2268518518518515E-3</v>
-      </c>
-      <c r="B51" s="4">
-        <v>6.9444444444444444E-5</v>
-      </c>
-      <c r="C51" s="38"/>
-      <c r="D51" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" s="5">
-        <f t="shared" si="3"/>
-        <v>6.2962962962962955E-3</v>
-      </c>
-      <c r="B52" s="4">
-        <v>6.9444444444444444E-5</v>
-      </c>
-      <c r="C52" s="37"/>
-      <c r="D52" s="32" t="s">
-        <v>22</v>
+      <c r="C52" s="21"/>
+      <c r="D52" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="49.5">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" s="5">
-        <f t="shared" si="3"/>
-        <v>6.3657407407407395E-3</v>
+        <f t="shared" si="4"/>
+        <v>6.6898148148148134E-3</v>
       </c>
       <c r="B53" s="4">
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C53" s="21"/>
+      <c r="C53" s="39" t="s">
+        <v>16</v>
+      </c>
       <c r="D53" s="6" t="s">
-        <v>142</v>
+        <v>36</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="33">
+        <v>102</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="132">
       <c r="A54" s="5">
-        <f t="shared" si="3"/>
-        <v>6.4814814814814804E-3</v>
+        <f t="shared" si="4"/>
+        <v>6.8055555555555543E-3</v>
       </c>
       <c r="B54" s="4">
-        <v>1.1574074074074073E-4</v>
-      </c>
-      <c r="C54" s="36" t="s">
-        <v>25</v>
-      </c>
+        <v>1.5046296296296294E-3</v>
+      </c>
+      <c r="C54" s="40"/>
       <c r="D54" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="132">
+        <v>34</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" s="5">
-        <f t="shared" si="3"/>
-        <v>6.5972222222222213E-3</v>
-      </c>
-      <c r="B55" s="4">
-        <v>1.5046296296296294E-3</v>
-      </c>
-      <c r="C55" s="37"/>
-      <c r="D55" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56" s="5">
-        <f t="shared" si="3"/>
-        <v>8.1018518518518514E-3</v>
-      </c>
-      <c r="C56" s="25" t="s">
-        <v>73</v>
+        <f t="shared" si="4"/>
+        <v>8.3101851851851843E-3</v>
+      </c>
+      <c r="C55" s="25" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="C4:C8"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="C42:C47"/>
-    <mergeCell ref="C31:C41"/>
-    <mergeCell ref="C48:C52"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C13:C30"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C41:C46"/>
+    <mergeCell ref="C30:C40"/>
+    <mergeCell ref="C47:C51"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="C14:C29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3477,7 +3469,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F25715-BEED-42F5-8F10-9FEA1FF7F5C3}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="4.83203125" bestFit="1" customWidth="1"/>
@@ -3486,16 +3478,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3503,10 +3495,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3514,10 +3506,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>121</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3525,10 +3517,21 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>120</v>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3547,18 +3550,18 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>123</v>
+        <v>88</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -3572,7 +3575,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -3586,7 +3589,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="B4">
         <v>6</v>

</xml_diff>